<commit_message>
added costs of jlc order
</commit_message>
<xml_diff>
--- a/manufacturing reports/BOM/BOM_xlsx-S001_additional_costs.xlsx
+++ b/manufacturing reports/BOM/BOM_xlsx-S001_additional_costs.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
   <si>
     <t>AN</t>
   </si>
@@ -137,13 +137,19 @@
     <t>RS</t>
   </si>
   <si>
-    <t>not sure</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>SN6501DBVR</t>
+  </si>
+  <si>
+    <t>win-source</t>
+  </si>
+  <si>
+    <t>Bestellung</t>
+  </si>
+  <si>
+    <t>Order #227370</t>
+  </si>
+  <si>
+    <t>win-source shipping</t>
   </si>
 </sst>
 </file>
@@ -177,7 +183,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -211,11 +217,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
@@ -226,6 +241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -506,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.08984375" customWidth="1"/>
@@ -514,12 +530,12 @@
     <col min="5" max="5" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -544,8 +560,11 @@
       <c r="H2" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -559,20 +578,23 @@
         <v>6</v>
       </c>
       <c r="E3" s="6">
-        <v>1</v>
+        <v>5.12</v>
       </c>
       <c r="F3" s="6">
         <f>E3*B3</f>
-        <v>2</v>
+        <v>10.24</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -599,7 +621,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -627,7 +649,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -655,7 +677,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -683,7 +705,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -710,7 +732,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -721,32 +743,60 @@
         <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E9" s="6">
-        <v>2.1800000000000002</v>
+        <f>8.23</f>
+        <v>8.23</v>
       </c>
       <c r="F9" s="6">
         <f t="shared" si="0"/>
-        <v>8.7200000000000006</v>
+        <v>32.92</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H9" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B10" s="7">
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="6">
+        <v>5</v>
+      </c>
+      <c r="F10" s="6">
+        <f t="shared" ref="F10" si="1">E10*B10</f>
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D11" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="6">
         <f>SUM(F3:F10)</f>
-        <v>158.19499999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>195.63499999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D13" s="5" t="s">
         <v>23</v>
       </c>
@@ -755,7 +805,7 @@
       </c>
       <c r="F13" s="6">
         <f>E13*F11</f>
-        <v>1581.9499999999998</v>
+        <v>1956.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>